<commit_message>
EDL au 09/09 - script rejets indus opérationnel pour SRR
</commit_message>
<xml_diff>
--- a/02_data/Liste fichiers.xlsx
+++ b/02_data/Liste fichiers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agencesdeleau.sharepoint.com/sites/AESN-Etudespressions/Shared Documents/Pressions/PANDA Pression/PANDA_Pression/02_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{9F15B30D-45CF-4112-AFE5-971E02649CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26AC7261-A766-4A2E-9673-9076B87450CB}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{9F15B30D-45CF-4112-AFE5-971E02649CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3342839F-C02C-4FDC-B352-EA6A67EF15C6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{64C32074-7079-410A-A620-303E49B92065}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{64C32074-7079-410A-A620-303E49B92065}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
   <si>
     <t>Dossier data</t>
   </si>
@@ -114,6 +114,12 @@
   </si>
   <si>
     <t>Table_Param_Unites.xlsx</t>
+  </si>
+  <si>
+    <t>Table_corresp_Roseau_Sitouref.xlsx</t>
+  </si>
+  <si>
+    <t>Tableau de correspondance entre Roseau et Sitouref, et entre SCL et STEP</t>
   </si>
 </sst>
 </file>
@@ -492,15 +498,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DFD6679-D3E2-41D9-A436-87DA488F4E33}">
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.21875" customWidth="1"/>
-    <col min="2" max="2" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="85.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="85.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -511,7 +517,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -522,7 +528,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -531,7 +537,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -542,7 +548,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -553,7 +559,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -564,7 +570,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -575,7 +581,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -586,7 +592,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -594,7 +600,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -602,7 +608,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -610,7 +616,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -619,24 +625,27 @@
         <v>22</v>
       </c>
     </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E0B707973A0EDF4D8C0132D38830BF56" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6fab73de96728382b95836a8b817e49f">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4222387a-a7c4-4a56-bf01-5dca1ac56634" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d5a3db95c4c940e29da1a6f70bc1044" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E0B707973A0EDF4D8C0132D38830BF56" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3aafe4bc97fbec4e49b652d28c2caa88">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4222387a-a7c4-4a56-bf01-5dca1ac56634" xmlns:ns3="a7b14cff-5e05-4f6c-b214-44a9052046af" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e93d2fa6853c901024a85aa72cf9a7fe" ns2:_="" ns3:_="">
     <xsd:import namespace="4222387a-a7c4-4a56-bf01-5dca1ac56634"/>
+    <xsd:import namespace="a7b14cff-5e05-4f6c-b214-44a9052046af"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -646,6 +655,11 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -670,6 +684,43 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2498e138-10ad-4e45-a616-48606944e53a" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a7b14cff-5e05-4f6c-b214-44a9052046af" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{e533d34c-d265-4360-97e9-dc06e3d45d14}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="a7b14cff-5e05-4f6c-b214-44a9052046af">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -771,13 +822,46 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <TaxCatchAll xmlns="a7b14cff-5e05-4f6c-b214-44a9052046af" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4222387a-a7c4-4a56-bf01-5dca1ac56634">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2ABD9C14-CA23-4916-8A4D-E6347A7223D3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4222387a-a7c4-4a56-bf01-5dca1ac56634"/>
+    <ds:schemaRef ds:uri="a7b14cff-5e05-4f6c-b214-44a9052046af"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6773EF1-3CA8-427C-B3DF-0D622DE2A109}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -785,15 +869,13 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{776A37C3-553D-4BD3-B115-DF7D653C6AF9}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{609A8DBE-E0F8-450C-90B7-A722ECCA9954}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a7b14cff-5e05-4f6c-b214-44a9052046af"/>
+    <ds:schemaRef ds:uri="4222387a-a7c4-4a56-bf01-5dca1ac56634"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>